<commit_message>
Finalize the data preparation
</commit_message>
<xml_diff>
--- a/data/processed/student_performance_cleaned.xlsx
+++ b/data/processed/student_performance_cleaned.xlsx
@@ -469,7 +469,7 @@
       </c>
       <c r="K1" t="inlineStr">
         <is>
-          <t>IT Total</t>
+          <t>Total IT Score</t>
         </is>
       </c>
       <c r="L1" t="inlineStr">
@@ -553,7 +553,9 @@
       <c r="J2" t="n">
         <v>46.49</v>
       </c>
-      <c r="K2" t="inlineStr"/>
+      <c r="K2" t="n">
+        <v>135</v>
+      </c>
       <c r="L2" t="n">
         <v>25.32</v>
       </c>
@@ -615,7 +617,9 @@
       <c r="J3" t="n">
         <v>44.33</v>
       </c>
-      <c r="K3" t="inlineStr"/>
+      <c r="K3" t="n">
+        <v>115</v>
+      </c>
       <c r="L3" t="n">
         <v>27.27</v>
       </c>
@@ -675,7 +679,9 @@
       <c r="J4" t="n">
         <v>44.96</v>
       </c>
-      <c r="K4" t="inlineStr"/>
+      <c r="K4" t="n">
+        <v>116</v>
+      </c>
       <c r="L4" t="n">
         <v>26.31</v>
       </c>
@@ -735,7 +741,9 @@
       <c r="J5" t="n">
         <v>42.14</v>
       </c>
-      <c r="K5" t="inlineStr"/>
+      <c r="K5" t="n">
+        <v>110</v>
+      </c>
       <c r="L5" t="n">
         <v>26.17</v>
       </c>
@@ -793,7 +801,9 @@
       <c r="J6" t="n">
         <v>41.8</v>
       </c>
-      <c r="K6" t="inlineStr"/>
+      <c r="K6" t="n">
+        <v>110</v>
+      </c>
       <c r="L6" t="n">
         <v>25.8</v>
       </c>
@@ -851,7 +861,9 @@
       <c r="J7" t="n">
         <v>41.6</v>
       </c>
-      <c r="K7" t="inlineStr"/>
+      <c r="K7" t="n">
+        <v>110</v>
+      </c>
       <c r="L7" t="n">
         <v>25.32</v>
       </c>
@@ -909,7 +921,9 @@
       <c r="J8" t="n">
         <v>44.61</v>
       </c>
-      <c r="K8" t="inlineStr"/>
+      <c r="K8" t="n">
+        <v>95</v>
+      </c>
       <c r="L8" t="n">
         <v>21.67</v>
       </c>
@@ -967,7 +981,9 @@
       <c r="J9" t="n">
         <v>40.71</v>
       </c>
-      <c r="K9" t="inlineStr"/>
+      <c r="K9" t="n">
+        <v>110</v>
+      </c>
       <c r="L9" t="n">
         <v>25.33</v>
       </c>
@@ -1025,7 +1041,9 @@
       <c r="J10" t="n">
         <v>42.31999999999999</v>
       </c>
-      <c r="K10" t="inlineStr"/>
+      <c r="K10" t="n">
+        <v>95</v>
+      </c>
       <c r="L10" t="n">
         <v>23.32</v>
       </c>
@@ -1083,7 +1101,9 @@
       <c r="J11" t="n">
         <v>39.65000000000001</v>
       </c>
-      <c r="K11" t="inlineStr"/>
+      <c r="K11" t="n">
+        <v>100</v>
+      </c>
       <c r="L11" t="n">
         <v>26.31</v>
       </c>
@@ -1141,7 +1161,9 @@
       <c r="J12" t="n">
         <v>46.23</v>
       </c>
-      <c r="K12" t="inlineStr"/>
+      <c r="K12" t="n">
+        <v>100</v>
+      </c>
       <c r="L12" t="n">
         <v>19.56</v>
       </c>
@@ -1205,7 +1227,9 @@
       <c r="J13" t="n">
         <v>44.19</v>
       </c>
-      <c r="K13" t="inlineStr"/>
+      <c r="K13" t="n">
+        <v>45</v>
+      </c>
       <c r="L13" t="n">
         <v>21.56</v>
       </c>
@@ -1263,7 +1287,9 @@
       <c r="J14" t="n">
         <v>40.73</v>
       </c>
-      <c r="K14" t="inlineStr"/>
+      <c r="K14" t="n">
+        <v>45</v>
+      </c>
       <c r="L14" t="n">
         <v>26.19</v>
       </c>
@@ -1325,7 +1351,9 @@
       <c r="J15" t="n">
         <v>38.71</v>
       </c>
-      <c r="K15" t="inlineStr"/>
+      <c r="K15" t="n">
+        <v>55</v>
+      </c>
       <c r="L15" t="n">
         <v>24.33</v>
       </c>
@@ -1383,7 +1411,9 @@
       <c r="J16" t="n">
         <v>37.59</v>
       </c>
-      <c r="K16" t="inlineStr"/>
+      <c r="K16" t="n">
+        <v>60</v>
+      </c>
       <c r="L16" t="n">
         <v>25.57</v>
       </c>
@@ -1441,7 +1471,9 @@
       <c r="J17" t="n">
         <v>38.36</v>
       </c>
-      <c r="K17" t="inlineStr"/>
+      <c r="K17" t="n">
+        <v>55</v>
+      </c>
       <c r="L17" t="n">
         <v>23.94</v>
       </c>
@@ -1499,7 +1531,9 @@
       <c r="J18" t="n">
         <v>38.45</v>
       </c>
-      <c r="K18" t="inlineStr"/>
+      <c r="K18" t="n">
+        <v>55</v>
+      </c>
       <c r="L18" t="n">
         <v>23.53</v>
       </c>
@@ -1557,7 +1591,9 @@
       <c r="J19" t="n">
         <v>41.37</v>
       </c>
-      <c r="K19" t="inlineStr"/>
+      <c r="K19" t="n">
+        <v>37.5</v>
+      </c>
       <c r="L19" t="n">
         <v>23.19</v>
       </c>
@@ -1619,7 +1655,9 @@
       <c r="J20" t="n">
         <v>37.05</v>
       </c>
-      <c r="K20" t="inlineStr"/>
+      <c r="K20" t="n">
+        <v>55</v>
+      </c>
       <c r="L20" t="n">
         <v>24.5</v>
       </c>
@@ -1677,7 +1715,9 @@
       <c r="J21" t="n">
         <v>35.84999999999999</v>
       </c>
-      <c r="K21" t="inlineStr"/>
+      <c r="K21" t="n">
+        <v>70</v>
+      </c>
       <c r="L21" t="n">
         <v>25.66</v>
       </c>
@@ -1735,7 +1775,9 @@
       <c r="J22" t="n">
         <v>34.69</v>
       </c>
-      <c r="K22" t="inlineStr"/>
+      <c r="K22" t="n">
+        <v>70</v>
+      </c>
       <c r="L22" t="n">
         <v>26.52</v>
       </c>
@@ -1793,7 +1835,9 @@
       <c r="J23" t="n">
         <v>45.1</v>
       </c>
-      <c r="K23" t="inlineStr"/>
+      <c r="K23" t="n">
+        <v>47.5</v>
+      </c>
       <c r="L23" t="n">
         <v>24.04</v>
       </c>
@@ -1857,7 +1901,9 @@
       <c r="J24" t="n">
         <v>39.2</v>
       </c>
-      <c r="K24" t="inlineStr"/>
+      <c r="K24" t="n">
+        <v>55</v>
+      </c>
       <c r="L24" t="n">
         <v>21.17</v>
       </c>
@@ -1915,7 +1961,9 @@
       <c r="J25" t="n">
         <v>37.34</v>
       </c>
-      <c r="K25" t="inlineStr"/>
+      <c r="K25" t="n">
+        <v>55</v>
+      </c>
       <c r="L25" t="n">
         <v>21.87</v>
       </c>
@@ -1973,7 +2021,9 @@
       <c r="J26" t="n">
         <v>34.52</v>
       </c>
-      <c r="K26" t="inlineStr"/>
+      <c r="K26" t="n">
+        <v>55</v>
+      </c>
       <c r="L26" t="n">
         <v>24.53</v>
       </c>
@@ -2031,7 +2081,9 @@
       <c r="J27" t="n">
         <v>40.87</v>
       </c>
-      <c r="K27" t="inlineStr"/>
+      <c r="K27" t="n">
+        <v>40</v>
+      </c>
       <c r="L27" t="n">
         <v>18.86</v>
       </c>
@@ -2089,7 +2141,9 @@
       <c r="J28" t="n">
         <v>35.07</v>
       </c>
-      <c r="K28" t="inlineStr"/>
+      <c r="K28" t="n">
+        <v>60</v>
+      </c>
       <c r="L28" t="n">
         <v>25.63</v>
       </c>
@@ -2147,7 +2201,9 @@
       <c r="J29" t="n">
         <v>34.66</v>
       </c>
-      <c r="K29" t="inlineStr"/>
+      <c r="K29" t="n">
+        <v>55</v>
+      </c>
       <c r="L29" t="n">
         <v>23.2</v>
       </c>
@@ -2205,7 +2261,9 @@
       <c r="J30" t="n">
         <v>32.22</v>
       </c>
-      <c r="K30" t="inlineStr"/>
+      <c r="K30" t="n">
+        <v>70</v>
+      </c>
       <c r="L30" t="n">
         <v>25.59</v>
       </c>
@@ -2263,7 +2321,9 @@
       <c r="J31" t="n">
         <v>41.89</v>
       </c>
-      <c r="K31" t="inlineStr"/>
+      <c r="K31" t="n">
+        <v>30</v>
+      </c>
       <c r="L31" t="n">
         <v>17.4</v>
       </c>
@@ -2321,7 +2381,9 @@
       <c r="J32" t="n">
         <v>35.56</v>
       </c>
-      <c r="K32" t="inlineStr"/>
+      <c r="K32" t="n">
+        <v>45</v>
+      </c>
       <c r="L32" t="n">
         <v>24.51</v>
       </c>
@@ -2379,7 +2441,9 @@
       <c r="J33" t="n">
         <v>38.3</v>
       </c>
-      <c r="K33" t="inlineStr"/>
+      <c r="K33" t="n">
+        <v>50</v>
+      </c>
       <c r="L33" t="n">
         <v>19.07</v>
       </c>
@@ -2437,7 +2501,9 @@
       <c r="J34" t="n">
         <v>33.57</v>
       </c>
-      <c r="K34" t="inlineStr"/>
+      <c r="K34" t="n">
+        <v>45</v>
+      </c>
       <c r="L34" t="n">
         <v>23.87</v>
       </c>
@@ -2495,7 +2561,9 @@
       <c r="J35" t="n">
         <v>37.40000000000001</v>
       </c>
-      <c r="K35" t="inlineStr"/>
+      <c r="K35" t="n">
+        <v>45</v>
+      </c>
       <c r="L35" t="n">
         <v>20.38</v>
       </c>
@@ -2553,7 +2621,9 @@
       <c r="J36" t="n">
         <v>36.83</v>
       </c>
-      <c r="K36" t="inlineStr"/>
+      <c r="K36" t="n">
+        <v>50</v>
+      </c>
       <c r="L36" t="n">
         <v>19.66</v>
       </c>
@@ -2611,7 +2681,9 @@
       <c r="J37" t="n">
         <v>39.69</v>
       </c>
-      <c r="K37" t="inlineStr"/>
+      <c r="K37" t="n">
+        <v>30</v>
+      </c>
       <c r="L37" t="n">
         <v>17.13</v>
       </c>
@@ -2669,7 +2741,9 @@
       <c r="J38" t="n">
         <v>34.97</v>
       </c>
-      <c r="K38" t="inlineStr"/>
+      <c r="K38" t="n">
+        <v>45</v>
+      </c>
       <c r="L38" t="n">
         <v>23.05</v>
       </c>
@@ -2727,7 +2801,9 @@
       <c r="J39" t="n">
         <v>36.02</v>
       </c>
-      <c r="K39" t="inlineStr"/>
+      <c r="K39" t="n">
+        <v>50</v>
+      </c>
       <c r="L39" t="n">
         <v>19.48</v>
       </c>
@@ -2785,7 +2861,9 @@
       <c r="J40" t="n">
         <v>31.47</v>
       </c>
-      <c r="K40" t="inlineStr"/>
+      <c r="K40" t="n">
+        <v>45</v>
+      </c>
       <c r="L40" t="n">
         <v>23.68</v>
       </c>
@@ -2843,7 +2921,9 @@
       <c r="J41" t="n">
         <v>36.65</v>
       </c>
-      <c r="K41" t="inlineStr"/>
+      <c r="K41" t="n">
+        <v>41</v>
+      </c>
       <c r="L41" t="n">
         <v>16.55</v>
       </c>
@@ -2903,7 +2983,9 @@
       <c r="J42" t="n">
         <v>33.24</v>
       </c>
-      <c r="K42" t="inlineStr"/>
+      <c r="K42" t="n">
+        <v>46</v>
+      </c>
       <c r="L42" t="n">
         <v>21.74</v>
       </c>
@@ -2963,7 +3045,9 @@
       <c r="J43" t="n">
         <v>34.41</v>
       </c>
-      <c r="K43" t="inlineStr"/>
+      <c r="K43" t="n">
+        <v>50</v>
+      </c>
       <c r="L43" t="n">
         <v>18.65</v>
       </c>
@@ -3021,7 +3105,9 @@
       <c r="J44" t="n">
         <v>30.07</v>
       </c>
-      <c r="K44" t="inlineStr"/>
+      <c r="K44" t="n">
+        <v>55</v>
+      </c>
       <c r="L44" t="n">
         <v>22.86</v>
       </c>
@@ -3079,7 +3165,9 @@
       <c r="J45" t="n">
         <v>33.07</v>
       </c>
-      <c r="K45" t="inlineStr"/>
+      <c r="K45" t="n">
+        <v>50</v>
+      </c>
       <c r="L45" t="n">
         <v>19.68</v>
       </c>
@@ -3137,7 +3225,9 @@
       <c r="J46" t="n">
         <v>36.1</v>
       </c>
-      <c r="K46" t="inlineStr"/>
+      <c r="K46" t="n">
+        <v>37.5</v>
+      </c>
       <c r="L46" t="n">
         <v>20.39</v>
       </c>
@@ -3199,7 +3289,9 @@
       <c r="J47" t="n">
         <v>33.82</v>
       </c>
-      <c r="K47" t="inlineStr"/>
+      <c r="K47" t="n">
+        <v>40</v>
+      </c>
       <c r="L47" t="n">
         <v>17.49</v>
       </c>
@@ -3257,7 +3349,9 @@
       <c r="J48" t="n">
         <v>30.58</v>
       </c>
-      <c r="K48" t="inlineStr"/>
+      <c r="K48" t="n">
+        <v>50</v>
+      </c>
       <c r="L48" t="n">
         <v>19.9</v>
       </c>
@@ -3315,7 +3409,9 @@
       <c r="J49" t="n">
         <v>35.71</v>
       </c>
-      <c r="K49" t="inlineStr"/>
+      <c r="K49" t="n">
+        <v>30</v>
+      </c>
       <c r="L49" t="n">
         <v>17.15</v>
       </c>
@@ -3377,7 +3473,9 @@
       <c r="J50" t="n">
         <v>33.2</v>
       </c>
-      <c r="K50" t="inlineStr"/>
+      <c r="K50" t="n">
+        <v>30</v>
+      </c>
       <c r="L50" t="n">
         <v>16.46</v>
       </c>
@@ -3435,7 +3533,9 @@
       <c r="J51" t="n">
         <v>23.64</v>
       </c>
-      <c r="K51" t="inlineStr"/>
+      <c r="K51" t="n">
+        <v>30</v>
+      </c>
       <c r="L51" t="n">
         <v>25.14</v>
       </c>
@@ -3497,7 +3597,9 @@
       <c r="J52" t="n">
         <v>29.72</v>
       </c>
-      <c r="K52" t="inlineStr"/>
+      <c r="K52" t="n">
+        <v>30</v>
+      </c>
       <c r="L52" t="n">
         <v>17.07</v>
       </c>
@@ -3559,7 +3661,9 @@
       <c r="J53" t="n">
         <v>27.31</v>
       </c>
-      <c r="K53" t="inlineStr"/>
+      <c r="K53" t="n">
+        <v>30</v>
+      </c>
       <c r="L53" t="n">
         <v>20</v>
       </c>
@@ -3621,7 +3725,9 @@
       <c r="J54" t="n">
         <v>30.8</v>
       </c>
-      <c r="K54" t="inlineStr"/>
+      <c r="K54" t="n">
+        <v>31</v>
+      </c>
       <c r="L54" t="n">
         <v>16.11</v>
       </c>
@@ -3681,7 +3787,9 @@
       <c r="J55" t="n">
         <v>27.34</v>
       </c>
-      <c r="K55" t="inlineStr"/>
+      <c r="K55" t="n">
+        <v>30</v>
+      </c>
       <c r="L55" t="n">
         <v>16.6</v>
       </c>
@@ -3743,7 +3851,9 @@
       <c r="J56" t="n">
         <v>25.59</v>
       </c>
-      <c r="K56" t="inlineStr"/>
+      <c r="K56" t="n">
+        <v>30</v>
+      </c>
       <c r="L56" t="n">
         <v>12.62</v>
       </c>
@@ -3805,7 +3915,9 @@
       <c r="J57" t="n">
         <v>26.62</v>
       </c>
-      <c r="K57" t="inlineStr"/>
+      <c r="K57" t="n">
+        <v>30</v>
+      </c>
       <c r="L57" t="n">
         <v>15</v>
       </c>
@@ -3869,7 +3981,9 @@
       <c r="J58" t="n">
         <v>45.34</v>
       </c>
-      <c r="K58" t="inlineStr"/>
+      <c r="K58" t="n">
+        <v>109.5</v>
+      </c>
       <c r="L58" t="n">
         <v>24.05</v>
       </c>
@@ -3929,7 +4043,9 @@
       <c r="J59" t="n">
         <v>40.75</v>
       </c>
-      <c r="K59" t="inlineStr"/>
+      <c r="K59" t="n">
+        <v>112</v>
+      </c>
       <c r="L59" t="n">
         <v>26.93</v>
       </c>
@@ -3991,7 +4107,9 @@
       <c r="J60" t="n">
         <v>43.73</v>
       </c>
-      <c r="K60" t="inlineStr"/>
+      <c r="K60" t="n">
+        <v>99.5</v>
+      </c>
       <c r="L60" t="n">
         <v>22.91</v>
       </c>
@@ -4051,7 +4169,9 @@
       <c r="J61" t="n">
         <v>40.72</v>
       </c>
-      <c r="K61" t="inlineStr"/>
+      <c r="K61" t="n">
+        <v>71</v>
+      </c>
       <c r="L61" t="n">
         <v>24.09</v>
       </c>
@@ -4119,7 +4239,9 @@
       <c r="J62" t="n">
         <v>47.4</v>
       </c>
-      <c r="K62" t="inlineStr"/>
+      <c r="K62" t="n">
+        <v>81</v>
+      </c>
       <c r="L62" t="n">
         <v>16.61</v>
       </c>
@@ -4185,7 +4307,9 @@
       <c r="J63" t="n">
         <v>40.49</v>
       </c>
-      <c r="K63" t="inlineStr"/>
+      <c r="K63" t="n">
+        <v>47</v>
+      </c>
       <c r="L63" t="n">
         <v>21.78</v>
       </c>
@@ -4245,7 +4369,9 @@
       <c r="J64" t="n">
         <v>39.95999999999999</v>
       </c>
-      <c r="K64" t="inlineStr"/>
+      <c r="K64" t="n">
+        <v>57</v>
+      </c>
       <c r="L64" t="n">
         <v>20.59</v>
       </c>
@@ -4305,7 +4431,9 @@
       <c r="J65" t="n">
         <v>38.38</v>
       </c>
-      <c r="K65" t="inlineStr"/>
+      <c r="K65" t="n">
+        <v>56</v>
+      </c>
       <c r="L65" t="n">
         <v>21.72</v>
       </c>
@@ -4367,7 +4495,9 @@
       <c r="J66" t="n">
         <v>40.99</v>
       </c>
-      <c r="K66" t="inlineStr"/>
+      <c r="K66" t="n">
+        <v>79</v>
+      </c>
       <c r="L66" t="n">
         <v>18.68</v>
       </c>
@@ -4427,7 +4557,9 @@
       <c r="J67" t="n">
         <v>36.39</v>
       </c>
-      <c r="K67" t="inlineStr"/>
+      <c r="K67" t="n">
+        <v>56</v>
+      </c>
       <c r="L67" t="n">
         <v>21.9</v>
       </c>
@@ -4489,7 +4621,9 @@
       <c r="J68" t="n">
         <v>34.72</v>
       </c>
-      <c r="K68" t="inlineStr"/>
+      <c r="K68" t="n">
+        <v>64</v>
+      </c>
       <c r="L68" t="n">
         <v>23.48</v>
       </c>
@@ -4549,7 +4683,9 @@
       <c r="J69" t="n">
         <v>34.72</v>
       </c>
-      <c r="K69" t="inlineStr"/>
+      <c r="K69" t="n">
+        <v>51</v>
+      </c>
       <c r="L69" t="n">
         <v>22.92</v>
       </c>
@@ -4611,7 +4747,9 @@
       <c r="J70" t="n">
         <v>34.05</v>
       </c>
-      <c r="K70" t="inlineStr"/>
+      <c r="K70" t="n">
+        <v>73</v>
+      </c>
       <c r="L70" t="n">
         <v>22.75</v>
       </c>
@@ -4671,7 +4809,9 @@
       <c r="J71" t="n">
         <v>40.66</v>
       </c>
-      <c r="K71" t="inlineStr"/>
+      <c r="K71" t="n">
+        <v>51</v>
+      </c>
       <c r="L71" t="n">
         <v>15.95</v>
       </c>
@@ -4737,7 +4877,9 @@
       <c r="J72" t="n">
         <v>35.61</v>
       </c>
-      <c r="K72" t="inlineStr"/>
+      <c r="K72" t="n">
+        <v>46</v>
+      </c>
       <c r="L72" t="n">
         <v>20.89</v>
       </c>
@@ -4797,7 +4939,9 @@
       <c r="J73" t="n">
         <v>32.38</v>
       </c>
-      <c r="K73" t="inlineStr"/>
+      <c r="K73" t="n">
+        <v>59</v>
+      </c>
       <c r="L73" t="n">
         <v>23.68</v>
       </c>
@@ -4859,7 +5003,9 @@
       <c r="J74" t="n">
         <v>34.96</v>
       </c>
-      <c r="K74" t="inlineStr"/>
+      <c r="K74" t="n">
+        <v>72</v>
+      </c>
       <c r="L74" t="n">
         <v>21.07</v>
       </c>
@@ -4919,7 +5065,9 @@
       <c r="J75" t="n">
         <v>34.01</v>
       </c>
-      <c r="K75" t="inlineStr"/>
+      <c r="K75" t="n">
+        <v>57</v>
+      </c>
       <c r="L75" t="n">
         <v>21.58</v>
       </c>
@@ -4981,7 +5129,9 @@
       <c r="J76" t="n">
         <v>32.72</v>
       </c>
-      <c r="K76" t="inlineStr"/>
+      <c r="K76" t="n">
+        <v>69.5</v>
+      </c>
       <c r="L76" t="n">
         <v>22.3</v>
       </c>
@@ -5043,7 +5193,9 @@
       <c r="J77" t="n">
         <v>36.06</v>
       </c>
-      <c r="K77" t="inlineStr"/>
+      <c r="K77" t="n">
+        <v>75</v>
+      </c>
       <c r="L77" t="n">
         <v>18.95</v>
       </c>
@@ -5103,7 +5255,9 @@
       <c r="J78" t="n">
         <v>35.7</v>
       </c>
-      <c r="K78" t="inlineStr"/>
+      <c r="K78" t="n">
+        <v>36</v>
+      </c>
       <c r="L78" t="n">
         <v>19.27</v>
       </c>
@@ -5169,7 +5323,9 @@
       <c r="J79" t="n">
         <v>40.61</v>
       </c>
-      <c r="K79" t="inlineStr"/>
+      <c r="K79" t="n">
+        <v>59</v>
+      </c>
       <c r="L79" t="n">
         <v>14.35</v>
       </c>
@@ -5235,7 +5391,9 @@
       <c r="J80" t="n">
         <v>30.53</v>
       </c>
-      <c r="K80" t="inlineStr"/>
+      <c r="K80" t="n">
+        <v>72.5</v>
+      </c>
       <c r="L80" t="n">
         <v>23.29</v>
       </c>
@@ -5297,7 +5455,9 @@
       <c r="J81" t="n">
         <v>34.92</v>
       </c>
-      <c r="K81" t="inlineStr"/>
+      <c r="K81" t="n">
+        <v>51</v>
+      </c>
       <c r="L81" t="n">
         <v>17.47</v>
       </c>
@@ -5357,7 +5517,9 @@
       <c r="J82" t="n">
         <v>27.68</v>
       </c>
-      <c r="K82" t="inlineStr"/>
+      <c r="K82" t="n">
+        <v>44.5</v>
+      </c>
       <c r="L82" t="n">
         <v>23.97</v>
       </c>
@@ -5421,7 +5583,9 @@
       <c r="J83" t="n">
         <v>34.59</v>
       </c>
-      <c r="K83" t="inlineStr"/>
+      <c r="K83" t="n">
+        <v>42</v>
+      </c>
       <c r="L83" t="n">
         <v>16.87</v>
       </c>
@@ -5481,7 +5645,9 @@
       <c r="J84" t="n">
         <v>24.6</v>
       </c>
-      <c r="K84" t="inlineStr"/>
+      <c r="K84" t="n">
+        <v>52</v>
+      </c>
       <c r="L84" t="n">
         <v>26.25</v>
       </c>
@@ -5547,7 +5713,9 @@
       <c r="J85" t="n">
         <v>25.47</v>
       </c>
-      <c r="K85" t="inlineStr"/>
+      <c r="K85" t="n">
+        <v>53</v>
+      </c>
       <c r="L85" t="n">
         <v>24.78</v>
       </c>
@@ -5611,7 +5779,9 @@
       <c r="J86" t="n">
         <v>26.62</v>
       </c>
-      <c r="K86" t="inlineStr"/>
+      <c r="K86" t="n">
+        <v>44.5</v>
+      </c>
       <c r="L86" t="n">
         <v>23.07</v>
       </c>
@@ -5675,7 +5845,9 @@
       <c r="J87" t="n">
         <v>35.02</v>
       </c>
-      <c r="K87" t="inlineStr"/>
+      <c r="K87" t="n">
+        <v>37</v>
+      </c>
       <c r="L87" t="n">
         <v>13.96</v>
       </c>
@@ -5739,7 +5911,9 @@
       <c r="J88" t="n">
         <v>24.82</v>
       </c>
-      <c r="K88" t="inlineStr"/>
+      <c r="K88" t="n">
+        <v>43.5</v>
+      </c>
       <c r="L88" t="n">
         <v>23.82</v>
       </c>
@@ -5805,7 +5979,9 @@
       <c r="J89" t="n">
         <v>35.42</v>
       </c>
-      <c r="K89" t="inlineStr"/>
+      <c r="K89" t="n">
+        <v>60</v>
+      </c>
       <c r="L89" t="n">
         <v>12.82</v>
       </c>
@@ -5869,7 +6045,9 @@
       <c r="J90" t="n">
         <v>26.54</v>
       </c>
-      <c r="K90" t="inlineStr"/>
+      <c r="K90" t="n">
+        <v>48.5</v>
+      </c>
       <c r="L90" t="n">
         <v>21.42</v>
       </c>
@@ -5935,7 +6113,9 @@
       <c r="J91" t="n">
         <v>26.19</v>
       </c>
-      <c r="K91" t="inlineStr"/>
+      <c r="K91" t="n">
+        <v>56.5</v>
+      </c>
       <c r="L91" t="n">
         <v>21.72</v>
       </c>
@@ -5999,7 +6179,9 @@
       <c r="J92" t="n">
         <v>31.54</v>
       </c>
-      <c r="K92" t="inlineStr"/>
+      <c r="K92" t="n">
+        <v>41</v>
+      </c>
       <c r="L92" t="n">
         <v>15.64</v>
       </c>
@@ -6059,7 +6241,9 @@
       <c r="J93" t="n">
         <v>22.57</v>
       </c>
-      <c r="K93" t="inlineStr"/>
+      <c r="K93" t="n">
+        <v>41.5</v>
+      </c>
       <c r="L93" t="n">
         <v>24.21</v>
       </c>
@@ -6125,7 +6309,9 @@
       <c r="J94" t="n">
         <v>25.08</v>
       </c>
-      <c r="K94" t="inlineStr"/>
+      <c r="K94" t="n">
+        <v>65.5</v>
+      </c>
       <c r="L94" t="n">
         <v>21.42</v>
       </c>
@@ -6191,7 +6377,9 @@
       <c r="J95" t="n">
         <v>30.01</v>
       </c>
-      <c r="K95" t="inlineStr"/>
+      <c r="K95" t="n">
+        <v>66</v>
+      </c>
       <c r="L95" t="n">
         <v>16.43</v>
       </c>
@@ -6251,7 +6439,9 @@
       <c r="J96" t="n">
         <v>24.69</v>
       </c>
-      <c r="K96" t="inlineStr"/>
+      <c r="K96" t="n">
+        <v>39.5</v>
+      </c>
       <c r="L96" t="n">
         <v>21.36</v>
       </c>
@@ -6317,7 +6507,9 @@
       <c r="J97" t="n">
         <v>29.82</v>
       </c>
-      <c r="K97" t="inlineStr"/>
+      <c r="K97" t="n">
+        <v>49.5</v>
+      </c>
       <c r="L97" t="n">
         <v>16.18</v>
       </c>
@@ -6381,7 +6573,9 @@
       <c r="J98" t="n">
         <v>29.45</v>
       </c>
-      <c r="K98" t="inlineStr"/>
+      <c r="K98" t="n">
+        <v>34</v>
+      </c>
       <c r="L98" t="n">
         <v>14.76</v>
       </c>
@@ -6447,7 +6641,9 @@
       <c r="J99" t="n">
         <v>27.57</v>
       </c>
-      <c r="K99" t="inlineStr"/>
+      <c r="K99" t="n">
+        <v>50</v>
+      </c>
       <c r="L99" t="n">
         <v>16.14</v>
       </c>
@@ -6511,7 +6707,9 @@
       <c r="J100" t="n">
         <v>25.04</v>
       </c>
-      <c r="K100" t="inlineStr"/>
+      <c r="K100" t="n">
+        <v>38</v>
+      </c>
       <c r="L100" t="n">
         <v>18.31</v>
       </c>
@@ -6577,7 +6775,9 @@
       <c r="J101" t="n">
         <v>21.07</v>
       </c>
-      <c r="K101" t="inlineStr"/>
+      <c r="K101" t="n">
+        <v>54.5</v>
+      </c>
       <c r="L101" t="n">
         <v>21.61</v>
       </c>
@@ -6643,7 +6843,9 @@
       <c r="J102" t="n">
         <v>27.23</v>
       </c>
-      <c r="K102" t="inlineStr"/>
+      <c r="K102" t="n">
+        <v>58</v>
+      </c>
       <c r="L102" t="n">
         <v>14.14</v>
       </c>
@@ -6707,7 +6909,9 @@
       <c r="J103" t="n">
         <v>23.06</v>
       </c>
-      <c r="K103" t="inlineStr"/>
+      <c r="K103" t="n">
+        <v>32</v>
+      </c>
       <c r="L103" t="n">
         <v>17.44</v>
       </c>
@@ -6773,7 +6977,9 @@
       <c r="J104" t="n">
         <v>22.43</v>
       </c>
-      <c r="K104" t="inlineStr"/>
+      <c r="K104" t="n">
+        <v>47.5</v>
+      </c>
       <c r="L104" t="n">
         <v>17.85</v>
       </c>
@@ -6839,7 +7045,9 @@
       <c r="J105" t="n">
         <v>25.56</v>
       </c>
-      <c r="K105" t="inlineStr"/>
+      <c r="K105" t="n">
+        <v>43.5</v>
+      </c>
       <c r="L105" t="n">
         <v>12.18</v>
       </c>
@@ -6903,7 +7111,9 @@
       <c r="J106" t="n">
         <v>21.58</v>
       </c>
-      <c r="K106" t="inlineStr"/>
+      <c r="K106" t="n">
+        <v>37</v>
+      </c>
       <c r="L106" t="n">
         <v>15.65</v>
       </c>
@@ -6967,7 +7177,9 @@
       <c r="J107" t="n">
         <v>20.47</v>
       </c>
-      <c r="K107" t="inlineStr"/>
+      <c r="K107" t="n">
+        <v>33</v>
+      </c>
       <c r="L107" t="n">
         <v>15.56</v>
       </c>
@@ -7033,7 +7245,9 @@
       <c r="J108" t="n">
         <v>18.69</v>
       </c>
-      <c r="K108" t="inlineStr"/>
+      <c r="K108" t="n">
+        <v>58</v>
+      </c>
       <c r="L108" t="n">
         <v>16.73</v>
       </c>
@@ -7099,7 +7313,9 @@
       <c r="J109" t="n">
         <v>24.56</v>
       </c>
-      <c r="K109" t="inlineStr"/>
+      <c r="K109" t="n">
+        <v>52</v>
+      </c>
       <c r="L109" t="n">
         <v>9.77</v>
       </c>
@@ -7165,7 +7381,9 @@
       <c r="J110" t="n">
         <v>20.34</v>
       </c>
-      <c r="K110" t="inlineStr"/>
+      <c r="K110" t="n">
+        <v>44.5</v>
+      </c>
       <c r="L110" t="n">
         <v>13.1</v>
       </c>
@@ -7229,7 +7447,9 @@
       <c r="J111" t="n">
         <v>19.41</v>
       </c>
-      <c r="K111" t="inlineStr"/>
+      <c r="K111" t="n">
+        <v>32</v>
+      </c>
       <c r="L111" t="n">
         <v>13.65</v>
       </c>
@@ -7293,7 +7513,9 @@
       <c r="J112" t="n">
         <v>17.93</v>
       </c>
-      <c r="K112" t="inlineStr"/>
+      <c r="K112" t="n">
+        <v>36</v>
+      </c>
       <c r="L112" t="n">
         <v>9.73</v>
       </c>
@@ -7357,7 +7579,9 @@
       <c r="J113" t="n">
         <v>48.56</v>
       </c>
-      <c r="K113" t="inlineStr"/>
+      <c r="K113" t="n">
+        <v>134</v>
+      </c>
       <c r="L113" t="n">
         <v>23.33</v>
       </c>
@@ -7417,7 +7641,9 @@
       <c r="J114" t="n">
         <v>49.28</v>
       </c>
-      <c r="K114" t="inlineStr"/>
+      <c r="K114" t="n">
+        <v>145</v>
+      </c>
       <c r="L114" t="n">
         <v>25.21</v>
       </c>
@@ -7477,7 +7703,9 @@
       <c r="J115" t="n">
         <v>51.11</v>
       </c>
-      <c r="K115" t="inlineStr"/>
+      <c r="K115" t="n">
+        <v>158</v>
+      </c>
       <c r="L115" t="n">
         <v>22.59</v>
       </c>
@@ -7539,7 +7767,9 @@
       <c r="J116" t="n">
         <v>49.87</v>
       </c>
-      <c r="K116" t="inlineStr"/>
+      <c r="K116" t="n">
+        <v>89.5</v>
+      </c>
       <c r="L116" t="n">
         <v>22.7</v>
       </c>
@@ -7603,7 +7833,9 @@
       <c r="J117" t="n">
         <v>49.81</v>
       </c>
-      <c r="K117" t="inlineStr"/>
+      <c r="K117" t="n">
+        <v>140</v>
+      </c>
       <c r="L117" t="n">
         <v>21.34</v>
       </c>
@@ -7663,7 +7895,9 @@
       <c r="J118" t="n">
         <v>50.11</v>
       </c>
-      <c r="K118" t="inlineStr"/>
+      <c r="K118" t="n">
+        <v>142</v>
+      </c>
       <c r="L118" t="n">
         <v>22</v>
       </c>
@@ -7723,7 +7957,9 @@
       <c r="J119" t="n">
         <v>49.46</v>
       </c>
-      <c r="K119" t="inlineStr"/>
+      <c r="K119" t="n">
+        <v>126</v>
+      </c>
       <c r="L119" t="n">
         <v>21.55</v>
       </c>
@@ -7783,7 +8019,9 @@
       <c r="J120" t="n">
         <v>49.14</v>
       </c>
-      <c r="K120" t="inlineStr"/>
+      <c r="K120" t="n">
+        <v>124</v>
+      </c>
       <c r="L120" t="n">
         <v>22.32</v>
       </c>
@@ -7843,7 +8081,9 @@
       <c r="J121" t="n">
         <v>54.56</v>
       </c>
-      <c r="K121" t="inlineStr"/>
+      <c r="K121" t="n">
+        <v>105</v>
+      </c>
       <c r="L121" t="n">
         <v>16.73</v>
       </c>
@@ -7903,7 +8143,9 @@
       <c r="J122" t="n">
         <v>51.29</v>
       </c>
-      <c r="K122" t="inlineStr"/>
+      <c r="K122" t="n">
+        <v>143</v>
+      </c>
       <c r="L122" t="n">
         <v>21.11</v>
       </c>
@@ -7963,7 +8205,9 @@
       <c r="J123" t="n">
         <v>49.28</v>
       </c>
-      <c r="K123" t="inlineStr"/>
+      <c r="K123" t="n">
+        <v>122</v>
+      </c>
       <c r="L123" t="n">
         <v>21.39</v>
       </c>
@@ -8023,7 +8267,9 @@
       <c r="J124" t="n">
         <v>53.19</v>
       </c>
-      <c r="K124" t="inlineStr"/>
+      <c r="K124" t="n">
+        <v>122</v>
+      </c>
       <c r="L124" t="n">
         <v>17.46</v>
       </c>
@@ -8083,7 +8329,9 @@
       <c r="J125" t="n">
         <v>50.88</v>
       </c>
-      <c r="K125" t="inlineStr"/>
+      <c r="K125" t="n">
+        <v>124</v>
+      </c>
       <c r="L125" t="n">
         <v>19.74</v>
       </c>
@@ -8143,7 +8391,9 @@
       <c r="J126" t="n">
         <v>48.29</v>
       </c>
-      <c r="K126" t="inlineStr"/>
+      <c r="K126" t="n">
+        <v>134</v>
+      </c>
       <c r="L126" t="n">
         <v>22.21</v>
       </c>
@@ -8203,7 +8453,9 @@
       <c r="J127" t="n">
         <v>49.49</v>
       </c>
-      <c r="K127" t="inlineStr"/>
+      <c r="K127" t="n">
+        <v>126</v>
+      </c>
       <c r="L127" t="n">
         <v>20.6</v>
       </c>
@@ -8263,7 +8515,9 @@
       <c r="J128" t="n">
         <v>49.66</v>
       </c>
-      <c r="K128" t="inlineStr"/>
+      <c r="K128" t="n">
+        <v>114</v>
+      </c>
       <c r="L128" t="n">
         <v>20.25</v>
       </c>
@@ -8323,7 +8577,9 @@
       <c r="J129" t="n">
         <v>52.13</v>
       </c>
-      <c r="K129" t="inlineStr"/>
+      <c r="K129" t="n">
+        <v>106</v>
+      </c>
       <c r="L129" t="n">
         <v>17.42</v>
       </c>
@@ -8383,7 +8639,9 @@
       <c r="J130" t="n">
         <v>50.38</v>
       </c>
-      <c r="K130" t="inlineStr"/>
+      <c r="K130" t="n">
+        <v>109</v>
+      </c>
       <c r="L130" t="n">
         <v>19.06</v>
       </c>
@@ -8443,7 +8701,9 @@
       <c r="J131" t="n">
         <v>49.46</v>
       </c>
-      <c r="K131" t="inlineStr"/>
+      <c r="K131" t="n">
+        <v>86</v>
+      </c>
       <c r="L131" t="n">
         <v>19.97</v>
       </c>
@@ -8503,7 +8763,9 @@
       <c r="J132" t="n">
         <v>52.38</v>
       </c>
-      <c r="K132" t="inlineStr"/>
+      <c r="K132" t="n">
+        <v>77</v>
+      </c>
       <c r="L132" t="n">
         <v>16.54</v>
       </c>
@@ -8563,7 +8825,9 @@
       <c r="J133" t="n">
         <v>48.91</v>
       </c>
-      <c r="K133" t="inlineStr"/>
+      <c r="K133" t="n">
+        <v>128</v>
+      </c>
       <c r="L133" t="n">
         <v>20.01</v>
       </c>
@@ -8623,7 +8887,9 @@
       <c r="J134" t="n">
         <v>51.63</v>
       </c>
-      <c r="K134" t="inlineStr"/>
+      <c r="K134" t="n">
+        <v>96</v>
+      </c>
       <c r="L134" t="n">
         <v>17.25</v>
       </c>
@@ -8683,7 +8949,9 @@
       <c r="J135" t="n">
         <v>50.38</v>
       </c>
-      <c r="K135" t="inlineStr"/>
+      <c r="K135" t="n">
+        <v>110</v>
+      </c>
       <c r="L135" t="n">
         <v>17.86</v>
       </c>
@@ -8743,7 +9011,9 @@
       <c r="J136" t="n">
         <v>48.63</v>
       </c>
-      <c r="K136" t="inlineStr"/>
+      <c r="K136" t="n">
+        <v>52</v>
+      </c>
       <c r="L136" t="n">
         <v>19.46</v>
       </c>
@@ -8803,7 +9073,9 @@
       <c r="J137" t="n">
         <v>48.66</v>
       </c>
-      <c r="K137" t="inlineStr"/>
+      <c r="K137" t="n">
+        <v>101</v>
+      </c>
       <c r="L137" t="n">
         <v>17.52</v>
       </c>
@@ -8863,7 +9135,9 @@
       <c r="J138" t="n">
         <v>49.63</v>
       </c>
-      <c r="K138" t="inlineStr"/>
+      <c r="K138" t="n">
+        <v>112</v>
+      </c>
       <c r="L138" t="n">
         <v>18.36</v>
       </c>
@@ -8923,7 +9197,9 @@
       <c r="J139" t="n">
         <v>52.94</v>
       </c>
-      <c r="K139" t="inlineStr"/>
+      <c r="K139" t="n">
+        <v>70</v>
+      </c>
       <c r="L139" t="n">
         <v>14.92</v>
       </c>
@@ -8987,7 +9263,9 @@
       <c r="J140" t="n">
         <v>52.56</v>
       </c>
-      <c r="K140" t="inlineStr"/>
+      <c r="K140" t="n">
+        <v>103</v>
+      </c>
       <c r="L140" t="n">
         <v>15.2</v>
       </c>
@@ -9047,7 +9325,9 @@
       <c r="J141" t="n">
         <v>49.44</v>
       </c>
-      <c r="K141" t="inlineStr"/>
+      <c r="K141" t="n">
+        <v>120</v>
+      </c>
       <c r="L141" t="n">
         <v>18.26</v>
       </c>
@@ -9107,7 +9387,9 @@
       <c r="J142" t="n">
         <v>49.81</v>
       </c>
-      <c r="K142" t="inlineStr"/>
+      <c r="K142" t="n">
+        <v>127</v>
+      </c>
       <c r="L142" t="n">
         <v>17.58</v>
       </c>
@@ -9167,7 +9449,9 @@
       <c r="J143" t="n">
         <v>52.81</v>
       </c>
-      <c r="K143" t="inlineStr"/>
+      <c r="K143" t="n">
+        <v>37</v>
+      </c>
       <c r="L143" t="n">
         <v>14.35</v>
       </c>
@@ -9227,7 +9511,9 @@
       <c r="J144" t="n">
         <v>48.93</v>
       </c>
-      <c r="K144" t="inlineStr"/>
+      <c r="K144" t="n">
+        <v>82</v>
+      </c>
       <c r="L144" t="n">
         <v>17.88</v>
       </c>
@@ -9287,7 +9573,9 @@
       <c r="J145" t="n">
         <v>46.78</v>
       </c>
-      <c r="K145" t="inlineStr"/>
+      <c r="K145" t="n">
+        <v>100</v>
+      </c>
       <c r="L145" t="n">
         <v>19.59</v>
       </c>
@@ -9351,7 +9639,9 @@
       <c r="J146" t="n">
         <v>47.41</v>
       </c>
-      <c r="K146" t="inlineStr"/>
+      <c r="K146" t="n">
+        <v>40</v>
+      </c>
       <c r="L146" t="n">
         <v>18.57</v>
       </c>
@@ -9415,7 +9705,9 @@
       <c r="J147" t="n">
         <v>53.69</v>
       </c>
-      <c r="K147" t="inlineStr"/>
+      <c r="K147" t="n">
+        <v>30</v>
+      </c>
       <c r="L147" t="n">
         <v>11.8</v>
       </c>
@@ -9479,7 +9771,9 @@
       <c r="J148" t="n">
         <v>48.91</v>
       </c>
-      <c r="K148" t="inlineStr"/>
+      <c r="K148" t="n">
+        <v>69</v>
+      </c>
       <c r="L148" t="n">
         <v>15.52</v>
       </c>
@@ -9539,7 +9833,9 @@
       <c r="J149" t="n">
         <v>54.44</v>
       </c>
-      <c r="K149" t="inlineStr"/>
+      <c r="K149" t="n">
+        <v>47</v>
+      </c>
       <c r="L149" t="n">
         <v>10.72</v>
       </c>
@@ -9603,7 +9899,9 @@
       <c r="J150" t="n">
         <v>48.16</v>
       </c>
-      <c r="K150" t="inlineStr"/>
+      <c r="K150" t="n">
+        <v>46</v>
+      </c>
       <c r="L150" t="n">
         <v>16.81</v>
       </c>
@@ -9663,7 +9961,9 @@
       <c r="J151" t="n">
         <v>50.53</v>
       </c>
-      <c r="K151" t="inlineStr"/>
+      <c r="K151" t="n">
+        <v>53</v>
+      </c>
       <c r="L151" t="n">
         <v>14.01</v>
       </c>
@@ -9729,7 +10029,9 @@
       <c r="J152" t="n">
         <v>51.16</v>
       </c>
-      <c r="K152" t="inlineStr"/>
+      <c r="K152" t="n">
+        <v>49</v>
+      </c>
       <c r="L152" t="n">
         <v>12.97</v>
       </c>
@@ -9793,7 +10095,9 @@
       <c r="J153" t="n">
         <v>49.78</v>
       </c>
-      <c r="K153" t="inlineStr"/>
+      <c r="K153" t="n">
+        <v>48</v>
+      </c>
       <c r="L153" t="n">
         <v>14.1</v>
       </c>
@@ -9857,7 +10161,9 @@
       <c r="J154" t="n">
         <v>53.44</v>
       </c>
-      <c r="K154" t="inlineStr"/>
+      <c r="K154" t="n">
+        <v>49</v>
+      </c>
       <c r="L154" t="n">
         <v>10.24</v>
       </c>
@@ -9921,7 +10227,9 @@
       <c r="J155" t="n">
         <v>47.41</v>
       </c>
-      <c r="K155" t="inlineStr"/>
+      <c r="K155" t="n">
+        <v>49</v>
+      </c>
       <c r="L155" t="n">
         <v>13.02</v>
       </c>
@@ -9985,7 +10293,9 @@
       <c r="J156" t="n">
         <v>48.56</v>
       </c>
-      <c r="K156" t="inlineStr"/>
+      <c r="K156" t="n">
+        <v>47</v>
+      </c>
       <c r="L156" t="n">
         <v>14.45</v>
       </c>
@@ -10049,7 +10359,9 @@
       <c r="J157" t="n">
         <v>51.38</v>
       </c>
-      <c r="K157" t="inlineStr"/>
+      <c r="K157" t="n">
+        <v>47</v>
+      </c>
       <c r="L157" t="n">
         <v>11.61</v>
       </c>
@@ -10115,7 +10427,9 @@
       <c r="J158" t="n">
         <v>47.98</v>
       </c>
-      <c r="K158" t="inlineStr"/>
+      <c r="K158" t="n">
+        <v>50</v>
+      </c>
       <c r="L158" t="n">
         <v>14.93</v>
       </c>
@@ -10179,7 +10493,9 @@
       <c r="J159" t="n">
         <v>50.11</v>
       </c>
-      <c r="K159" t="inlineStr"/>
+      <c r="K159" t="n">
+        <v>56</v>
+      </c>
       <c r="L159" t="n">
         <v>12.86</v>
       </c>
@@ -10243,7 +10559,9 @@
       <c r="J160" t="n">
         <v>50.53</v>
       </c>
-      <c r="K160" t="inlineStr"/>
+      <c r="K160" t="n">
+        <v>49</v>
+      </c>
       <c r="L160" t="n">
         <v>11.62</v>
       </c>
@@ -10307,7 +10625,9 @@
       <c r="J161" t="n">
         <v>47.41</v>
       </c>
-      <c r="K161" t="inlineStr"/>
+      <c r="K161" t="n">
+        <v>46</v>
+      </c>
       <c r="L161" t="n">
         <v>13.37</v>
       </c>
@@ -10371,7 +10691,9 @@
       <c r="J162" t="n">
         <v>49.39</v>
       </c>
-      <c r="K162" t="inlineStr"/>
+      <c r="K162" t="n">
+        <v>52</v>
+      </c>
       <c r="L162" t="n">
         <v>10.67</v>
       </c>
@@ -10435,7 +10757,9 @@
       <c r="J163" t="n">
         <v>48.79</v>
       </c>
-      <c r="K163" t="inlineStr"/>
+      <c r="K163" t="n">
+        <v>49</v>
+      </c>
       <c r="L163" t="n">
         <v>10.9</v>
       </c>
@@ -10499,7 +10823,9 @@
       <c r="J164" t="n">
         <v>48.71</v>
       </c>
-      <c r="K164" t="inlineStr"/>
+      <c r="K164" t="n">
+        <v>48</v>
+      </c>
       <c r="L164" t="n">
         <v>10.09</v>
       </c>
@@ -10563,7 +10889,9 @@
       <c r="J165" t="n">
         <v>47.28</v>
       </c>
-      <c r="K165" t="inlineStr"/>
+      <c r="K165" t="n">
+        <v>37</v>
+      </c>
       <c r="L165" t="n">
         <v>9.76</v>
       </c>
@@ -10627,7 +10955,9 @@
       <c r="J166" t="n">
         <v>48.56</v>
       </c>
-      <c r="K166" t="inlineStr"/>
+      <c r="K166" t="n">
+        <v>52</v>
+      </c>
       <c r="L166" t="n">
         <v>8.130000000000001</v>
       </c>
@@ -10691,7 +11021,9 @@
       <c r="J167" t="n">
         <v>81.81</v>
       </c>
-      <c r="K167" t="inlineStr"/>
+      <c r="K167" t="n">
+        <v>142</v>
+      </c>
       <c r="L167" t="inlineStr"/>
       <c r="M167" t="n">
         <v>10</v>
@@ -10751,7 +11083,9 @@
       <c r="J168" t="n">
         <v>81.56</v>
       </c>
-      <c r="K168" t="inlineStr"/>
+      <c r="K168" t="n">
+        <v>104</v>
+      </c>
       <c r="L168" t="inlineStr"/>
       <c r="M168" t="n">
         <v>10</v>
@@ -10809,7 +11143,9 @@
       <c r="J169" t="n">
         <v>81.06</v>
       </c>
-      <c r="K169" t="inlineStr"/>
+      <c r="K169" t="n">
+        <v>102</v>
+      </c>
       <c r="L169" t="inlineStr"/>
       <c r="M169" t="n">
         <v>10</v>
@@ -10867,7 +11203,9 @@
       <c r="J170" t="n">
         <v>80.31</v>
       </c>
-      <c r="K170" t="inlineStr"/>
+      <c r="K170" t="n">
+        <v>102</v>
+      </c>
       <c r="L170" t="inlineStr"/>
       <c r="M170" t="n">
         <v>10</v>
@@ -10925,7 +11263,9 @@
       <c r="J171" t="n">
         <v>79.95999999999999</v>
       </c>
-      <c r="K171" t="inlineStr"/>
+      <c r="K171" t="n">
+        <v>102</v>
+      </c>
       <c r="L171" t="inlineStr"/>
       <c r="M171" t="n">
         <v>10</v>
@@ -10983,7 +11323,9 @@
       <c r="J172" t="n">
         <v>79.81</v>
       </c>
-      <c r="K172" t="inlineStr"/>
+      <c r="K172" t="n">
+        <v>101</v>
+      </c>
       <c r="L172" t="inlineStr"/>
       <c r="M172" t="n">
         <v>10</v>
@@ -11041,7 +11383,9 @@
       <c r="J173" t="n">
         <v>79.81</v>
       </c>
-      <c r="K173" t="inlineStr"/>
+      <c r="K173" t="n">
+        <v>96</v>
+      </c>
       <c r="L173" t="inlineStr"/>
       <c r="M173" t="n">
         <v>10</v>
@@ -11099,7 +11443,9 @@
       <c r="J174" t="n">
         <v>79.84999999999999</v>
       </c>
-      <c r="K174" t="inlineStr"/>
+      <c r="K174" t="n">
+        <v>94</v>
+      </c>
       <c r="L174" t="inlineStr"/>
       <c r="M174" t="n">
         <v>9.800000000000001</v>
@@ -11157,7 +11503,9 @@
       <c r="J175" t="n">
         <v>80.81</v>
       </c>
-      <c r="K175" t="inlineStr"/>
+      <c r="K175" t="n">
+        <v>108</v>
+      </c>
       <c r="L175" t="inlineStr"/>
       <c r="M175" t="n">
         <v>8.5</v>
@@ -11217,7 +11565,9 @@
       <c r="J176" t="n">
         <v>79.95</v>
       </c>
-      <c r="K176" t="inlineStr"/>
+      <c r="K176" t="n">
+        <v>85</v>
+      </c>
       <c r="L176" t="inlineStr"/>
       <c r="M176" t="n">
         <v>9.25</v>
@@ -11275,7 +11625,9 @@
       <c r="J177" t="n">
         <v>79.09999999999999</v>
       </c>
-      <c r="K177" t="inlineStr"/>
+      <c r="K177" t="n">
+        <v>102</v>
+      </c>
       <c r="L177" t="inlineStr"/>
       <c r="M177" t="n">
         <v>10</v>
@@ -11333,7 +11685,9 @@
       <c r="J178" t="n">
         <v>79.06</v>
       </c>
-      <c r="K178" t="inlineStr"/>
+      <c r="K178" t="n">
+        <v>97</v>
+      </c>
       <c r="L178" t="inlineStr"/>
       <c r="M178" t="n">
         <v>10</v>
@@ -11391,7 +11745,9 @@
       <c r="J179" t="n">
         <v>78.97</v>
       </c>
-      <c r="K179" t="inlineStr"/>
+      <c r="K179" t="n">
+        <v>95</v>
+      </c>
       <c r="L179" t="inlineStr"/>
       <c r="M179" t="n">
         <v>10</v>
@@ -11449,7 +11805,9 @@
       <c r="J180" t="n">
         <v>78.83</v>
       </c>
-      <c r="K180" t="inlineStr"/>
+      <c r="K180" t="n">
+        <v>101</v>
+      </c>
       <c r="L180" t="inlineStr"/>
       <c r="M180" t="n">
         <v>10</v>
@@ -11507,7 +11865,9 @@
       <c r="J181" t="n">
         <v>78.7</v>
       </c>
-      <c r="K181" t="inlineStr"/>
+      <c r="K181" t="n">
+        <v>105</v>
+      </c>
       <c r="L181" t="inlineStr"/>
       <c r="M181" t="n">
         <v>10</v>
@@ -11565,7 +11925,9 @@
       <c r="J182" t="n">
         <v>78.7</v>
       </c>
-      <c r="K182" t="inlineStr"/>
+      <c r="K182" t="n">
+        <v>102</v>
+      </c>
       <c r="L182" t="inlineStr"/>
       <c r="M182" t="n">
         <v>10</v>
@@ -11623,7 +11985,9 @@
       <c r="J183" t="n">
         <v>78.59999999999999</v>
       </c>
-      <c r="K183" t="inlineStr"/>
+      <c r="K183" t="n">
+        <v>101</v>
+      </c>
       <c r="L183" t="inlineStr"/>
       <c r="M183" t="n">
         <v>10</v>
@@ -11681,7 +12045,9 @@
       <c r="J184" t="n">
         <v>78.58</v>
       </c>
-      <c r="K184" t="inlineStr"/>
+      <c r="K184" t="n">
+        <v>105</v>
+      </c>
       <c r="L184" t="inlineStr"/>
       <c r="M184" t="n">
         <v>10</v>
@@ -11739,7 +12105,9 @@
       <c r="J185" t="n">
         <v>78.55</v>
       </c>
-      <c r="K185" t="inlineStr"/>
+      <c r="K185" t="n">
+        <v>106</v>
+      </c>
       <c r="L185" t="inlineStr"/>
       <c r="M185" t="n">
         <v>10</v>
@@ -11797,7 +12165,9 @@
       <c r="J186" t="n">
         <v>78.53</v>
       </c>
-      <c r="K186" t="inlineStr"/>
+      <c r="K186" t="n">
+        <v>105</v>
+      </c>
       <c r="L186" t="inlineStr"/>
       <c r="M186" t="n">
         <v>10</v>
@@ -11855,7 +12225,9 @@
       <c r="J187" t="n">
         <v>79.84999999999999</v>
       </c>
-      <c r="K187" t="inlineStr"/>
+      <c r="K187" t="n">
+        <v>108</v>
+      </c>
       <c r="L187" t="inlineStr"/>
       <c r="M187" t="n">
         <v>8.5</v>
@@ -11915,7 +12287,9 @@
       <c r="J188" t="n">
         <v>79.08</v>
       </c>
-      <c r="K188" t="inlineStr"/>
+      <c r="K188" t="n">
+        <v>89</v>
+      </c>
       <c r="L188" t="inlineStr"/>
       <c r="M188" t="n">
         <v>9.25</v>
@@ -11973,7 +12347,9 @@
       <c r="J189" t="n">
         <v>78.33</v>
       </c>
-      <c r="K189" t="inlineStr"/>
+      <c r="K189" t="n">
+        <v>96</v>
+      </c>
       <c r="L189" t="inlineStr"/>
       <c r="M189" t="n">
         <v>10</v>
@@ -12031,7 +12407,9 @@
       <c r="J190" t="n">
         <v>79.95</v>
       </c>
-      <c r="K190" t="inlineStr"/>
+      <c r="K190" t="n">
+        <v>90</v>
+      </c>
       <c r="L190" t="inlineStr"/>
       <c r="M190" t="n">
         <v>8.25</v>
@@ -12089,7 +12467,9 @@
       <c r="J191" t="n">
         <v>77.97</v>
       </c>
-      <c r="K191" t="inlineStr"/>
+      <c r="K191" t="n">
+        <v>96</v>
+      </c>
       <c r="L191" t="inlineStr"/>
       <c r="M191" t="n">
         <v>10</v>
@@ -12147,7 +12527,9 @@
       <c r="J192" t="n">
         <v>78.59999999999999</v>
       </c>
-      <c r="K192" t="inlineStr"/>
+      <c r="K192" t="n">
+        <v>95</v>
+      </c>
       <c r="L192" t="inlineStr"/>
       <c r="M192" t="n">
         <v>9.25</v>
@@ -12205,7 +12587,9 @@
       <c r="J193" t="n">
         <v>78.45</v>
       </c>
-      <c r="K193" t="inlineStr"/>
+      <c r="K193" t="n">
+        <v>95</v>
+      </c>
       <c r="L193" t="inlineStr"/>
       <c r="M193" t="n">
         <v>9.25</v>
@@ -12263,7 +12647,9 @@
       <c r="J194" t="n">
         <v>78.34999999999999</v>
       </c>
-      <c r="K194" t="inlineStr"/>
+      <c r="K194" t="n">
+        <v>113</v>
+      </c>
       <c r="L194" t="inlineStr"/>
       <c r="M194" t="n">
         <v>9.25</v>
@@ -12323,7 +12709,9 @@
       <c r="J195" t="n">
         <v>79.83</v>
       </c>
-      <c r="K195" t="inlineStr"/>
+      <c r="K195" t="n">
+        <v>93</v>
+      </c>
       <c r="L195" t="inlineStr"/>
       <c r="M195" t="n">
         <v>7.75</v>
@@ -12381,7 +12769,9 @@
       <c r="J196" t="n">
         <v>77.45</v>
       </c>
-      <c r="K196" t="inlineStr"/>
+      <c r="K196" t="n">
+        <v>103</v>
+      </c>
       <c r="L196" t="inlineStr"/>
       <c r="M196" t="n">
         <v>10</v>
@@ -12439,7 +12829,9 @@
       <c r="J197" t="n">
         <v>77.05</v>
       </c>
-      <c r="K197" t="inlineStr"/>
+      <c r="K197" t="n">
+        <v>107</v>
+      </c>
       <c r="L197" t="inlineStr"/>
       <c r="M197" t="n">
         <v>10</v>
@@ -12497,7 +12889,9 @@
       <c r="J198" t="n">
         <v>76.73</v>
       </c>
-      <c r="K198" t="inlineStr"/>
+      <c r="K198" t="n">
+        <v>103</v>
+      </c>
       <c r="L198" t="inlineStr"/>
       <c r="M198" t="n">
         <v>10</v>
@@ -12555,7 +12949,9 @@
       <c r="J199" t="n">
         <v>76.7</v>
       </c>
-      <c r="K199" t="inlineStr"/>
+      <c r="K199" t="n">
+        <v>141</v>
+      </c>
       <c r="L199" t="inlineStr"/>
       <c r="M199" t="n">
         <v>10</v>
@@ -12615,7 +13011,9 @@
       <c r="J200" t="n">
         <v>76.59999999999999</v>
       </c>
-      <c r="K200" t="inlineStr"/>
+      <c r="K200" t="n">
+        <v>98</v>
+      </c>
       <c r="L200" t="inlineStr"/>
       <c r="M200" t="n">
         <v>10</v>
@@ -12673,7 +13071,9 @@
       <c r="J201" t="n">
         <v>77.34999999999999</v>
       </c>
-      <c r="K201" t="inlineStr"/>
+      <c r="K201" t="n">
+        <v>95</v>
+      </c>
       <c r="L201" t="inlineStr"/>
       <c r="M201" t="n">
         <v>9.15</v>
@@ -12731,7 +13131,9 @@
       <c r="J202" t="n">
         <v>76.15000000000001</v>
       </c>
-      <c r="K202" t="inlineStr"/>
+      <c r="K202" t="n">
+        <v>104</v>
+      </c>
       <c r="L202" t="inlineStr"/>
       <c r="M202" t="n">
         <v>10</v>
@@ -12789,7 +13191,9 @@
       <c r="J203" t="n">
         <v>77.95999999999999</v>
       </c>
-      <c r="K203" t="inlineStr"/>
+      <c r="K203" t="n">
+        <v>91</v>
+      </c>
       <c r="L203" t="inlineStr"/>
       <c r="M203" t="n">
         <v>8.15</v>
@@ -12847,7 +13251,9 @@
       <c r="J204" t="n">
         <v>76.72</v>
       </c>
-      <c r="K204" t="inlineStr"/>
+      <c r="K204" t="n">
+        <v>86</v>
+      </c>
       <c r="L204" t="inlineStr"/>
       <c r="M204" t="n">
         <v>9.25</v>
@@ -12905,7 +13311,9 @@
       <c r="J205" t="n">
         <v>75.78</v>
       </c>
-      <c r="K205" t="inlineStr"/>
+      <c r="K205" t="n">
+        <v>102</v>
+      </c>
       <c r="L205" t="inlineStr"/>
       <c r="M205" t="n">
         <v>10</v>
@@ -12963,7 +13371,9 @@
       <c r="J206" t="n">
         <v>75.73</v>
       </c>
-      <c r="K206" t="inlineStr"/>
+      <c r="K206" t="n">
+        <v>107</v>
+      </c>
       <c r="L206" t="inlineStr"/>
       <c r="M206" t="n">
         <v>10</v>
@@ -13021,7 +13431,9 @@
       <c r="J207" t="n">
         <v>75.62</v>
       </c>
-      <c r="K207" t="inlineStr"/>
+      <c r="K207" t="n">
+        <v>102</v>
+      </c>
       <c r="L207" t="inlineStr"/>
       <c r="M207" t="n">
         <v>10</v>
@@ -13079,7 +13491,9 @@
       <c r="J208" t="n">
         <v>78.20999999999999</v>
       </c>
-      <c r="K208" t="inlineStr"/>
+      <c r="K208" t="n">
+        <v>88</v>
+      </c>
       <c r="L208" t="inlineStr"/>
       <c r="M208" t="n">
         <v>7.4</v>
@@ -13137,7 +13551,9 @@
       <c r="J209" t="n">
         <v>76.09999999999999</v>
       </c>
-      <c r="K209" t="inlineStr"/>
+      <c r="K209" t="n">
+        <v>99</v>
+      </c>
       <c r="L209" t="inlineStr"/>
       <c r="M209" t="n">
         <v>9.5</v>
@@ -13197,7 +13613,9 @@
       <c r="J210" t="n">
         <v>75.48</v>
       </c>
-      <c r="K210" t="inlineStr"/>
+      <c r="K210" t="n">
+        <v>102</v>
+      </c>
       <c r="L210" t="inlineStr"/>
       <c r="M210" t="n">
         <v>10</v>
@@ -13255,7 +13673,9 @@
       <c r="J211" t="n">
         <v>78.40000000000001</v>
       </c>
-      <c r="K211" t="inlineStr"/>
+      <c r="K211" t="n">
+        <v>90</v>
+      </c>
       <c r="L211" t="inlineStr"/>
       <c r="M211" t="n">
         <v>7</v>
@@ -13313,7 +13733,9 @@
       <c r="J212" t="n">
         <v>75.27</v>
       </c>
-      <c r="K212" t="inlineStr"/>
+      <c r="K212" t="n">
+        <v>138</v>
+      </c>
       <c r="L212" t="inlineStr"/>
       <c r="M212" t="n">
         <v>10</v>
@@ -13373,7 +13795,9 @@
       <c r="J213" t="n">
         <v>74.63</v>
       </c>
-      <c r="K213" t="inlineStr"/>
+      <c r="K213" t="n">
+        <v>97</v>
+      </c>
       <c r="L213" t="inlineStr"/>
       <c r="M213" t="n">
         <v>10</v>
@@ -13431,7 +13855,9 @@
       <c r="J214" t="n">
         <v>75.95</v>
       </c>
-      <c r="K214" t="inlineStr"/>
+      <c r="K214" t="n">
+        <v>85</v>
+      </c>
       <c r="L214" t="inlineStr"/>
       <c r="M214" t="n">
         <v>8.5</v>
@@ -13489,7 +13915,9 @@
       <c r="J215" t="n">
         <v>74.97</v>
       </c>
-      <c r="K215" t="inlineStr"/>
+      <c r="K215" t="n">
+        <v>88</v>
+      </c>
       <c r="L215" t="inlineStr"/>
       <c r="M215" t="n">
         <v>9.25</v>
@@ -13547,7 +13975,9 @@
       <c r="J216" t="n">
         <v>74.90000000000001</v>
       </c>
-      <c r="K216" t="inlineStr"/>
+      <c r="K216" t="n">
+        <v>85</v>
+      </c>
       <c r="L216" t="inlineStr"/>
       <c r="M216" t="n">
         <v>8.5</v>
@@ -13605,7 +14035,9 @@
       <c r="J217" t="n">
         <v>74.65000000000001</v>
       </c>
-      <c r="K217" t="inlineStr"/>
+      <c r="K217" t="n">
+        <v>86</v>
+      </c>
       <c r="L217" t="inlineStr"/>
       <c r="M217" t="n">
         <v>8.25</v>
@@ -13663,7 +14095,9 @@
       <c r="J218" t="n">
         <v>74.5</v>
       </c>
-      <c r="K218" t="inlineStr"/>
+      <c r="K218" t="n">
+        <v>88</v>
+      </c>
       <c r="L218" t="inlineStr"/>
       <c r="M218" t="n">
         <v>8.15</v>
@@ -13721,7 +14155,9 @@
       <c r="J219" t="n">
         <v>74.31999999999999</v>
       </c>
-      <c r="K219" t="inlineStr"/>
+      <c r="K219" t="n">
+        <v>84</v>
+      </c>
       <c r="L219" t="inlineStr"/>
       <c r="M219" t="n">
         <v>8</v>

</xml_diff>